<commit_message>
al the design for the begin and the data as have to be
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -13,10 +13,10 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1789264819" val="1234" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1789264819" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1789264819" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1789264819"/>
+      <pm:revision xmlns:pm="smNativeData" day="1789947624" val="1234" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1789947624" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1789947624" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1789947624"/>
     </ext>
   </extLst>
 </workbook>
@@ -130,7 +130,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1789264819" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1789947624" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -145,7 +145,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1789264819" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1789947624" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -161,7 +161,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1789264819" fgClr="0563C1" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1789947624" fgClr="0563C1" ulstyle="single" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -177,7 +177,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1789264819" fgClr="0563C1" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1789947624" fgClr="0563C1" ulstyle="single" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -194,7 +194,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1789264819" fgClr="0563C1" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1789947624" fgClr="0563C1" ulstyle="single" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -211,7 +211,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1789264819" fgClr="0563C1" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1789947624" fgClr="0563C1" ulstyle="single" kern="1">
             <pm:latin face="Calibri" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -234,7 +234,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1789264819" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1789947624" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -256,7 +256,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1789264819"/>
+          <pm:border xmlns:pm="smNativeData" id="1789947624"/>
         </ext>
       </extLst>
     </border>
@@ -275,7 +275,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1789264819"/>
+          <pm:border xmlns:pm="smNativeData" id="1789947624"/>
         </ext>
       </extLst>
     </border>
@@ -313,10 +313,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1789264819" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1789947624" count="1">
         <pm:charStyle name="Normal" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1789264819" count="1">
+      <pm:colors xmlns:pm="smNativeData" id="1789947624" count="1">
         <pm:color name="Color 24" rgb="0563C1"/>
       </pm:colors>
     </ext>
@@ -790,7 +790,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1789264819" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1789947624" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -799,16 +799,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1789264819" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1789264819" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1789264819" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1789264819" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1789947624" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1789947624" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1789947624" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1789947624" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1789264819" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1789947624" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>